<commit_message>
Oct 2026: agrega Jonny Lam (aviso entrada 14/10/2026)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hd1sTjd8iyWuDeJNNhaqX
</commit_message>
<xml_diff>
--- a/Control_Contratistas_2026.xlsx
+++ b/Control_Contratistas_2026.xlsx
@@ -8440,17 +8440,24 @@
         <f>MAESTRO!C9</f>
         <v/>
       </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E9" s="13" t="inlineStr"/>
-      <c r="F9" s="12">
+      <c r="D9" s="20" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E9" s="21" t="n">
+        <v>46309</v>
+      </c>
+      <c r="F9" s="20">
         <f>IF(D9="SI","✔ ACCESO","✘ SIN ACCESO")</f>
         <v/>
       </c>
-      <c r="G9" s="13" t="inlineStr"/>
+      <c r="G9" s="22" t="inlineStr">
+        <is>
+          <t>• Lam Gamboa Jonny Segundo
+(Aviso de Entrada — Quevedo | 14/10/2026)</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="5" t="n">
@@ -9114,17 +9121,24 @@
         <f>MAESTRO!C9</f>
         <v/>
       </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E9" s="13" t="inlineStr"/>
-      <c r="F9" s="12">
+      <c r="D9" s="20" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E9" s="21" t="n">
+        <v>46309</v>
+      </c>
+      <c r="F9" s="20">
         <f>IF(D9="SI","✔ ACCESO","✘ SIN ACCESO")</f>
         <v/>
       </c>
-      <c r="G9" s="13" t="inlineStr"/>
+      <c r="G9" s="22" t="inlineStr">
+        <is>
+          <t>• Lam Gamboa Jonny Segundo
+(Aviso de Entrada — Quevedo | 14/10/2026)</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="5" t="n">

</xml_diff>

<commit_message>
Oct 2026: agrega Industrias Don Quiño / Dailer (16/10/2026, 9 trabajadores)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hd1sTjd8iyWuDeJNNhaqX
</commit_message>
<xml_diff>
--- a/Control_Contratistas_2026.xlsx
+++ b/Control_Contratistas_2026.xlsx
@@ -1959,7 +1959,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="18" customHeight="1">
+    <row r="6" ht="117" customHeight="1">
       <c r="A6" s="5" t="n">
         <v>2</v>
       </c>
@@ -1971,17 +1971,32 @@
         <f>MAESTRO!C6</f>
         <v/>
       </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E6" s="14" t="inlineStr"/>
-      <c r="F6" s="12">
+      <c r="D6" s="20" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E6" s="21" t="n">
+        <v>46311</v>
+      </c>
+      <c r="F6" s="20">
         <f>IF(D6="SI","✔ ACCESO","✘ SIN ACCESO")</f>
         <v/>
       </c>
-      <c r="G6" s="14" t="inlineStr"/>
+      <c r="G6" s="23" t="inlineStr">
+        <is>
+          <t>• Aguilar Valverde Dubert Uwaldo
+• Palma Macias Leandro Wladimir
+• Quiñonez Garcia Dixon Antonio
+• Romero Cegido Jorge Luis
+• Quiñonez Garcia Dailer Fernando
+• Arguello Medina Wilmer Ricardo
+• Cabrera Cabrera Juan Pablo
+• Cabrera Rodriguez Angel Andres
+• Mendoza Suarez Neicer Armando
+(Planilla IESS período 2026-09 + 4 Avisos de Entrada (05/10 y 16/10))</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="78" customHeight="1">
       <c r="A7" s="7" t="n">

</xml_diff>

<commit_message>
Oct 2026: agrega Meta technologie/D-NETSOF (07/10/2026, 2 trabajadores)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hd1sTjd8iyWuDeJNNhaqX
</commit_message>
<xml_diff>
--- a/Control_Contratistas_2026.xlsx
+++ b/Control_Contratistas_2026.xlsx
@@ -2291,7 +2291,7 @@
       </c>
       <c r="G17" s="13" t="inlineStr"/>
     </row>
-    <row r="18" ht="18" customHeight="1">
+    <row r="18" ht="26" customHeight="1">
       <c r="A18" s="5" t="n">
         <v>14</v>
       </c>
@@ -2303,17 +2303,25 @@
         <f>MAESTRO!C18</f>
         <v/>
       </c>
-      <c r="D18" s="12" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E18" s="14" t="inlineStr"/>
-      <c r="F18" s="12">
+      <c r="D18" s="20" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E18" s="21" t="n">
+        <v>46302</v>
+      </c>
+      <c r="F18" s="20">
         <f>IF(D18="SI","✔ ACCESO","✘ SIN ACCESO")</f>
         <v/>
       </c>
-      <c r="G18" s="14" t="inlineStr"/>
+      <c r="G18" s="23" t="inlineStr">
+        <is>
+          <t>• Pluas Fajardo Orly Enrique
+• Davila Giler Jhon Michael
+(D-NETSOF | Avisos de Entrada 07/10/2026)</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="65" customHeight="1">
       <c r="A19" s="7" t="n">

</xml_diff>

<commit_message>
Oct 2026: agrega Víctor Andrade Calderón (19/10/2026, 11 trabajadores)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012hd1sTjd8iyWuDeJNNhaqX
</commit_message>
<xml_diff>
--- a/Control_Contratistas_2026.xlsx
+++ b/Control_Contratistas_2026.xlsx
@@ -2089,7 +2089,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1">
+    <row r="10" ht="143" customHeight="1">
       <c r="A10" s="5" t="n">
         <v>6</v>
       </c>
@@ -2101,17 +2101,34 @@
         <f>MAESTRO!C10</f>
         <v/>
       </c>
-      <c r="D10" s="12" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E10" s="14" t="inlineStr"/>
-      <c r="F10" s="12">
+      <c r="D10" s="20" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="E10" s="21" t="n">
+        <v>46314</v>
+      </c>
+      <c r="F10" s="20">
         <f>IF(D10="SI","✔ ACCESO","✘ SIN ACCESO")</f>
         <v/>
       </c>
-      <c r="G10" s="14" t="inlineStr"/>
+      <c r="G10" s="23" t="inlineStr">
+        <is>
+          <t>• Andrade Calderon Victor Volivar
+• Angulo Preciado Jhon Enrique
+• Barclay Suarez Jose Carlos
+• Beltran Jimenez Walter Oswaldo
+• Gonzalez Aviles Jonathan Stalin
+• Lozada Palacios Adrian Anibal
+• Navarrete Navarrete Luis Alejandro
+• Rocafuerte Alvarado Alex Jairo
+• Sandoval Rivera Jose Luis
+• Velez Mure Juan Carlos
+• Villamar Chevez Mauricio Damian
+(Período 2026-09)</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="7" t="n">

</xml_diff>